<commit_message>
Catalogue sprint: fresh blind accuracy test after grouping pass (identity/grouping ~99% adjudicated)
20 new releases, 84 pins; automatic identity 94%, grouping 97%, edition 87%, date 90%;
hand-adjudicated identity and grouping ~99%. Two source disagreements recorded and now
blocked for review. Scorer: accent folding, release-date dimension, generic-word fixes.
Pilot unchanged (100 pins / 23 pages), reloads offline. 42 tests pass, audit clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
+++ b/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
@@ -10165,7 +10165,7 @@
         <v>0</v>
       </c>
       <c r="J86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K86" t="s">
         <v>849</v>
@@ -15972,7 +15972,7 @@
         <v>0</v>
       </c>
       <c r="J219">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K219" t="s">
         <v>850</v>

</xml_diff>

<commit_message>
Catalogue engine: canonical edition types (removes 11 false conflicts); sprint STATUS check-in
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
+++ b/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
@@ -10684,7 +10684,7 @@
         <v>0</v>
       </c>
       <c r="J98">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K98" t="s">
         <v>849</v>
@@ -14696,7 +14696,7 @@
         <v>0</v>
       </c>
       <c r="J190">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K190" t="s">
         <v>850</v>
@@ -15136,7 +15136,7 @@
         <v>2</v>
       </c>
       <c r="J200">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K200" t="s">
         <v>850</v>
@@ -16101,7 +16101,7 @@
         <v>4</v>
       </c>
       <c r="J222">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K222" t="s">
         <v>850</v>
@@ -18119,7 +18119,7 @@
         <v>0</v>
       </c>
       <c r="J268">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K268" t="s">
         <v>850</v>
@@ -19835,7 +19835,7 @@
         <v>1</v>
       </c>
       <c r="J307">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K307" t="s">
         <v>850</v>

</xml_diff>

<commit_message>
Catalogue engine: review-hold rule; 8 possible EPCOT duplicates blocked until reviewed; STATUS priorities
Holds come from evidence/99_review_holds.json (maintainer instruction) and make the pins
unapprovable (conflict). Next actions now prioritise #241 and the first 100 verified,
imported staging pins over new candidates. 45 tests pass, audit clean, pilot reloads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
+++ b/research/catalogue-engine/out/consolidated/verification_worklist.xlsx
@@ -10415,7 +10415,7 @@
         <v>3</v>
       </c>
       <c r="J91">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K91" t="s">
         <v>853</v>
@@ -10717,7 +10717,7 @@
         <v>0</v>
       </c>
       <c r="J98">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K98" t="s">
         <v>853</v>

</xml_diff>